<commit_message>
refactor: 아티팩트 Description 추가 업데이트
</commit_message>
<xml_diff>
--- a/Assets/Data/Excel/Artifacts.xlsx
+++ b/Assets/Data/Excel/Artifacts.xlsx
@@ -596,7 +596,7 @@
       </c>
       <c r="C3" s="0" t="inlineStr">
         <is>
-          <t>아군 마법사 클래스의 방어력이 3 증가</t>
+          <t xml:space="preserve">마법사 계열 아군의 방어력이 3 증가</t>
         </is>
       </c>
       <c r="D3" s="0" t="inlineStr">
@@ -671,7 +671,7 @@
       </c>
       <c r="C6" s="0" t="inlineStr">
         <is>
-          <t>건물의 골드 생산 보상이 지급될 때마다 기본 지급량이 3 증가</t>
+          <t xml:space="preserve">건물에서 골드를 생산할 때마다 기본 생산량이 3 증가</t>
         </is>
       </c>
       <c r="D6" s="0" t="inlineStr">
@@ -721,7 +721,7 @@
       </c>
       <c r="C8" s="0" t="inlineStr">
         <is>
-          <t>아군 궁수 클래스의 최대 체력이 8% 증가</t>
+          <t xml:space="preserve">궁수 계열 아군의 최대 체력이 8% 증가</t>
         </is>
       </c>
       <c r="D8" s="0" t="inlineStr">
@@ -746,7 +746,8 @@
       </c>
       <c r="C9" s="0" t="inlineStr">
         <is>
-          <t>아군 전체의 기본 공격 배율이 80% 증가하고 스킬 배율이 40% 감소. 스킬 배율을 사용하는 회복량에도 적용</t>
+          <t xml:space="preserve">아군 전체의 기본 공격 배율이 80% 증가하고 스킬 배율이 40% 감소
+스킬 배율에 영향을 받는 회복량도 함께 감소</t>
         </is>
       </c>
       <c r="D9" s="0" t="inlineStr">
@@ -771,7 +772,7 @@
       </c>
       <c r="C10" s="0" t="inlineStr">
         <is>
-          <t>아군 검사 클래스의 이동속도와 탐지 범위가 15% 증가</t>
+          <t xml:space="preserve">검사 계열 아군의 이동속도와 탐지 범위가 15% 증가</t>
         </is>
       </c>
       <c r="D10" s="0" t="inlineStr">
@@ -846,7 +847,7 @@
       </c>
       <c r="C13" s="0" t="inlineStr">
         <is>
-          <t>아군 전사 클래스의 방어력이 3 증가</t>
+          <t xml:space="preserve">전사 계열 아군의 방어력이 3 증가</t>
         </is>
       </c>
       <c r="D13" s="0" t="inlineStr">
@@ -921,7 +922,7 @@
       </c>
       <c r="C16" s="0" t="inlineStr">
         <is>
-          <t>아군 검사 클래스의 기본 공격 배율이 8% 증가</t>
+          <t xml:space="preserve">검사 계열 아군의 기본 공격 배율이 8% 증가</t>
         </is>
       </c>
       <c r="D16" s="0" t="inlineStr">
@@ -971,7 +972,7 @@
       </c>
       <c r="C18" s="0" t="inlineStr">
         <is>
-          <t>아군 궁수 클래스의 치명타 확률이 2% 증가</t>
+          <t xml:space="preserve">궁수 계열 아군의 치명타 확률이 2% 증가</t>
         </is>
       </c>
       <c r="D18" s="0" t="inlineStr">
@@ -1046,7 +1047,7 @@
       </c>
       <c r="C21" s="0" t="inlineStr">
         <is>
-          <t>아군 전사 클래스가 받는 피해 배율이 8% 감소</t>
+          <t xml:space="preserve">전사 계열 아군이 받는 피해 배율이 8% 감소</t>
         </is>
       </c>
       <c r="D21" s="0" t="inlineStr">
@@ -1071,7 +1072,7 @@
       </c>
       <c r="C22" s="0" t="inlineStr">
         <is>
-          <t>아군 검사 클래스의 공격속도가 12% 증가</t>
+          <t xml:space="preserve">검사 계열 아군의 공격속도가 12% 증가</t>
         </is>
       </c>
       <c r="D22" s="0" t="inlineStr">
@@ -1096,7 +1097,7 @@
       </c>
       <c r="C23" s="0" t="inlineStr">
         <is>
-          <t>아군 마법사 클래스의 스킬 배율이 15% 증가</t>
+          <t xml:space="preserve">마법사 계열 아군의 스킬 배율이 15% 증가</t>
         </is>
       </c>
       <c r="D23" s="0" t="inlineStr">
@@ -1121,7 +1122,7 @@
       </c>
       <c r="C24" s="0" t="inlineStr">
         <is>
-          <t>아군 마법사 클래스의 쿨다운 감소율이 5% 증가</t>
+          <t xml:space="preserve">마법사 계열 아군의 쿨다운 감소율이 5% 증가</t>
         </is>
       </c>
       <c r="D24" s="0" t="inlineStr">
@@ -1146,7 +1147,7 @@
       </c>
       <c r="C25" s="0" t="inlineStr">
         <is>
-          <t>아군 궁수 클래스의 방어력 무시 비율이 8% 증가</t>
+          <t xml:space="preserve">궁수 계열 아군의 방어력 무시 비율이 8% 증가</t>
         </is>
       </c>
       <c r="D25" s="0" t="inlineStr">
@@ -1171,7 +1172,7 @@
       </c>
       <c r="C26" s="0" t="inlineStr">
         <is>
-          <t>아군 검사 클래스의 흡혈 비율이 3% 증가</t>
+          <t xml:space="preserve">검사 계열 아군의 흡혈 비율이 3% 증가</t>
         </is>
       </c>
       <c r="D26" s="0" t="inlineStr">
@@ -1221,7 +1222,7 @@
       </c>
       <c r="C28" s="0" t="inlineStr">
         <is>
-          <t>아군 궁수 클래스의 치명타 피해 배율이 20% 증가</t>
+          <t xml:space="preserve">궁수 계열 아군의 치명타 피해 배율이 20% 증가</t>
         </is>
       </c>
       <c r="D28" s="0" t="inlineStr">
@@ -1546,7 +1547,7 @@
       </c>
       <c r="C41" s="0" t="inlineStr">
         <is>
-          <t>아군 마법사 클래스의 스킬 배율이 70%, 쿨다운 감소율이 15% 증가하고 최대 체력이 40% 감소</t>
+          <t xml:space="preserve">마법사 계열 아군의 스킬 배율이 70%, 쿨다운 감소율이 15% 증가하고 최대 체력이 40% 감소</t>
         </is>
       </c>
       <c r="D41" s="0" t="inlineStr">
@@ -1596,7 +1597,8 @@
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>아군 유닛의 체력이 처음 25% 이하가 되면 자신의 최대 체력의 15%만큼 회복. 유닛마다 1회 발동</t>
+          <t xml:space="preserve">아군 유닛의 체력이 처음 25% 이하로 떨어지면 자신의 최대 체력의 15%만큼 회복
+유닛당 1회 발동</t>
         </is>
       </c>
       <c r="D43" s="0" t="inlineStr">
@@ -1621,7 +1623,7 @@
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>아군 마법사 클래스가 액티브 스킬 사용을 완료하면 자신의 최대 체력의 5%만큼 보호막 획득</t>
+          <t xml:space="preserve">마법사 계열 아군이 액티브 스킬 사용을 마치면 자신의 최대 체력의 5%만큼 보호막 획득</t>
         </is>
       </c>
       <c r="D44" s="0" t="inlineStr">
@@ -1646,7 +1648,8 @@
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>아군 전사 클래스는 자신 주변 반경 2에 적이 3명 이상 있으면 공격속도가 20% 증가. 조건은 0.5초마다 확인</t>
+          <t xml:space="preserve">전사 계열 아군은 주변 반경 2 안에 적이 3명 이상 있으면 공격속도가 20% 증가
+0.5초마다 갱신</t>
         </is>
       </c>
       <c r="D45" s="0" t="inlineStr">
@@ -1696,7 +1699,8 @@
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>아군 검사 클래스는 자신 주변 반경 2에 적이 정확히 1명 있으면 주는 피해가 20% 증가. 조건은 0.5초마다 확인</t>
+          <t xml:space="preserve">검사 계열 아군은 주변 반경 2 안에 적이 1명만 있으면 주는 피해가 20% 증가
+0.5초마다 갱신</t>
         </is>
       </c>
       <c r="D47" s="0" t="inlineStr">
@@ -1721,7 +1725,8 @@
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>아군 전사 클래스가 액티브 스킬 사용을 완료하면 4초 동안 이동속도가 15% 증가. 다시 발동하면 지속시간만 갱신</t>
+          <t xml:space="preserve">전사 계열 아군이 액티브 스킬 사용을 마치면 4초 동안 이동속도가 15% 증가
+중첩되지 않으며 재발동 시 지속시간 갱신</t>
         </is>
       </c>
       <c r="D48" s="0" t="inlineStr">
@@ -1746,7 +1751,7 @@
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>아군 궁수 클래스가 액티브 스킬 사용을 완료하면 자신 주변 반경 16의 가까운 적 최대 3명에게 각각 공격력의 50%에 해당하는 물리 피해를 주는 추가 투사체 발사</t>
+          <t xml:space="preserve">궁수 계열 아군이 액티브 스킬 사용을 마치면 주변 반경 16 안의 가까운 적 최대 3명에게 추가 투사체를 발사해 각각 공격력의 50%만큼 물리 피해를 줌</t>
         </is>
       </c>
       <c r="D49" s="0" t="inlineStr">
@@ -1771,7 +1776,7 @@
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>아군 궁수 클래스는 체력이 80% 이상이면 공격력이 15% 증가</t>
+          <t xml:space="preserve">궁수 계열 아군은 체력이 80% 이상일 때 공격력이 15% 증가</t>
         </is>
       </c>
       <c r="D50" s="0" t="inlineStr">
@@ -1796,7 +1801,7 @@
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>아군 1티어 유닛은 체력이 50% 이하이면 공격력이 25% 증가</t>
+          <t xml:space="preserve">아군 1티어 유닛은 체력이 50% 이하일 때 공격력이 25% 증가</t>
         </is>
       </c>
       <c r="D51" s="0" t="inlineStr">
@@ -1821,7 +1826,8 @@
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>아군 마법사 클래스가 액티브 스킬 사용을 완료하면 자신 주변 반경 8의 적 최대 3명의 이동속도가 4초 동안 30% 감소. 다시 발동하면 지속시간만 갱신</t>
+          <t xml:space="preserve">마법사 계열 아군이 액티브 스킬 사용을 마치면 주변 반경 8 안의 적 최대 3명의 이동속도를 4초 동안 30% 감소시킴
+중첩되지 않으며 재발동 시 지속시간 갱신</t>
         </is>
       </c>
       <c r="D52" s="0" t="inlineStr">
@@ -1846,7 +1852,7 @@
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>아군 광신도 클래스가 액티브 스킬 사용을 완료하면 자신 주변 반경 3의 다른 아군 최대 3명에게 자신의 최대 체력의 8%만큼 보호막 부여</t>
+          <t xml:space="preserve">광신도 계열 아군이 액티브 스킬 사용을 마치면 주변 반경 3 안의 다른 아군 최대 3명에게 자신의 최대 체력의 8%만큼 보호막 부여</t>
         </is>
       </c>
       <c r="D53" s="0" t="inlineStr">
@@ -1871,7 +1877,7 @@
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>아군 광신도 클래스는 자신 주변 반경 3에 다른 아군이 1명 이상 있으면 주는 회복량과 보호막량이 20% 증가</t>
+          <t xml:space="preserve">광신도 계열 아군은 주변 반경 3 안에 다른 아군이 1명 이상 있으면 주는 회복량과 보호막량이 20% 증가</t>
         </is>
       </c>
       <c r="D54" s="0" t="inlineStr">
@@ -1921,7 +1927,7 @@
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>아군 마법사 클래스가 액티브 스킬 사용을 완료하면 자신의 최대 체력의 2%만큼 회복</t>
+          <t xml:space="preserve">마법사 계열 아군이 액티브 스킬 사용을 마치면 자신의 최대 체력의 2%만큼 회복</t>
         </is>
       </c>
       <c r="D56" s="0" t="inlineStr">
@@ -1946,7 +1952,8 @@
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>아군 궁수 클래스가 적을 처치하면 4초 동안 공격력이 10% 증가. 다시 발동하면 지속시간만 갱신</t>
+          <t xml:space="preserve">궁수 계열 아군이 적을 처치하면 4초 동안 공격력이 10% 증가
+중첩되지 않으며 재발동 시 지속시간 갱신</t>
         </is>
       </c>
       <c r="D57" s="0" t="inlineStr">
@@ -1971,7 +1978,8 @@
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>아군 전사 클래스가 액티브 스킬 사용을 완료하면 5초 동안 받는 피해가 20% 감소. 다시 발동하면 지속시간만 갱신</t>
+          <t xml:space="preserve">전사 계열 아군이 액티브 스킬 사용을 마치면 5초 동안 받는 피해가 20% 감소
+중첩되지 않으며 재발동 시 지속시간 갱신</t>
         </is>
       </c>
       <c r="D58" s="0" t="inlineStr">
@@ -1996,7 +2004,7 @@
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>아군 검사 클래스가 액티브 스킬 사용을 완료하면 자신 주변 반경 5의 가까운 적 최대 2명에게 각각 공격력의 75%에 해당하는 추가 물리 피해</t>
+          <t xml:space="preserve">검사 계열 아군이 액티브 스킬 사용을 마치면 주변 반경 5 안의 가까운 적 최대 2명에게 각각 공격력의 75%만큼 추가 물리 피해를 줌</t>
         </is>
       </c>
       <c r="D59" s="0" t="inlineStr">
@@ -2021,7 +2029,7 @@
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>광전사는 체력이 60% 이하이면 받는 회복량과 보호막량이 50% 증가</t>
+          <t xml:space="preserve">광전사는 체력이 60% 이하일 때 받는 회복량과 보호막량이 50% 증가</t>
         </is>
       </c>
       <c r="D60" s="0" t="inlineStr">
@@ -2046,7 +2054,8 @@
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>저격수의 체력이 처음 40% 이하가 되면 자신의 최대 체력의 40%만큼 보호막 획득. 유닛마다 1회 발동</t>
+          <t xml:space="preserve">저격수의 체력이 처음 40% 이하로 떨어지면 자신의 최대 체력의 40%만큼 보호막 획득
+유닛당 1회 발동</t>
         </is>
       </c>
       <c r="D61" s="0" t="inlineStr">
@@ -2071,7 +2080,8 @@
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>아군 1티어 유닛이 처음 액티브 스킬 사용을 시작하면 20초 동안 공격속도가 40% 증가. 유닛마다 1회 발동</t>
+          <t xml:space="preserve">아군 1티어 유닛이 첫 액티브 스킬을 사용하기 시작하면 20초 동안 공격속도가 40% 증가
+유닛당 1회 발동</t>
         </is>
       </c>
       <c r="D62" s="0" t="inlineStr">
@@ -2096,7 +2106,8 @@
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>아군 전사 클래스는 체력이 50% 이하이면 공격속도가 75% 증가. 체력과 관계없이 받는 피해가 20% 증가</t>
+          <t xml:space="preserve">전사 계열 아군은 체력이 50% 이하일 때 공격속도가 75% 증가
+받는 피해는 항상 20% 증가</t>
         </is>
       </c>
       <c r="D63" s="0" t="inlineStr">
@@ -2121,7 +2132,9 @@
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>아군 검사 클래스가 액티브 스킬 사용을 완료하면 5초 동안 공격속도가 60% 증가. 다시 발동하면 지속시간만 갱신. 받는 회복량과 보호막량은 항상 30% 감소</t>
+          <t xml:space="preserve">검사 계열 아군이 액티브 스킬 사용을 마치면 5초 동안 공격속도가 60% 증가
+중첩되지 않으며 재발동 시 지속시간 갱신
+받는 회복량과 보호막량은 항상 30% 감소</t>
         </is>
       </c>
       <c r="D64" s="0" t="inlineStr">
@@ -2146,7 +2159,8 @@
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>아군 궁수 클래스가 액티브 스킬 사용을 완료하면 자신 주변 반경 16의 가까운 적 최대 4명에게 각각 공격력의 100%에 해당하는 물리 피해를 주는 추가 투사체 발사. 공격력은 항상 10% 감소</t>
+          <t xml:space="preserve">궁수 계열 아군이 액티브 스킬 사용을 마치면 주변 반경 16 안의 가까운 적 최대 4명에게 추가 투사체를 발사해 각각 공격력의 100%만큼 물리 피해를 줌
+공격력은 항상 10% 감소</t>
         </is>
       </c>
       <c r="D65" s="0" t="inlineStr">
@@ -2171,7 +2185,8 @@
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>아군 광신도 클래스가 6초마다 자신 주변 반경 3의 다른 아군 최대 3명의 체력을 각각 자신의 최대 체력의 15%만큼 회복. 자신의 최대 체력은 20% 감소</t>
+          <t xml:space="preserve">광신도 계열 아군이 6초마다 주변 반경 3 안의 다른 아군 최대 3명을 자신의 최대 체력의 15%만큼 각각 회복
+자신의 최대 체력은 20% 감소</t>
         </is>
       </c>
       <c r="D66" s="0" t="inlineStr">
@@ -2196,7 +2211,7 @@
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>아군 유닛은 6초마다 자신의 체력이 50% 이하이면 최대 체력의 2%만큼 회복</t>
+          <t xml:space="preserve">아군 유닛이 6초마다 체력이 50% 이하인 경우 자신의 최대 체력의 2%만큼 회복</t>
         </is>
       </c>
       <c r="D67" s="0" t="inlineStr">
@@ -2221,7 +2236,8 @@
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>아군 검사 클래스가 적을 처치하면 3초 동안 이동속도가 12% 증가. 다시 발동하면 지속시간 갱신</t>
+          <t xml:space="preserve">검사 계열 아군이 적을 처치하면 3초 동안 이동속도가 12% 증가
+재발동 시 지속시간 갱신</t>
         </is>
       </c>
       <c r="D68" s="0" t="inlineStr">
@@ -2246,7 +2262,7 @@
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>장궁수가 액티브 스킬 사용을 완료하면 자신 주변 반경 6의 적 최대 2명을 0.7초 동안 속박</t>
+          <t xml:space="preserve">장궁수가 액티브 스킬 사용을 마치면 주변 반경 6 안의 적 최대 2명을 0.7초 동안 속박</t>
         </is>
       </c>
       <c r="D69" s="0" t="inlineStr">
@@ -2271,7 +2287,8 @@
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>아군 검사 클래스가 피해를 줄 때마다 4초 동안 공격력이 3% 증가하며 최대 5회 중첩. 다시 발동하면 지속시간 갱신</t>
+          <t xml:space="preserve">검사 계열 아군이 피해를 줄 때마다 4초 동안 공격력이 3% 증가
+최대 5회 중첩되며 재발동 시 지속시간 갱신</t>
         </is>
       </c>
       <c r="D70" s="0" t="inlineStr">
@@ -2296,7 +2313,7 @@
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>아군 궁수 클래스는 자신 주변 반경 3에 다른 아군이 없으면 공격력이 18% 증가</t>
+          <t xml:space="preserve">궁수 계열 아군은 주변 반경 3 안에 다른 아군이 없으면 공격력이 18% 증가</t>
         </is>
       </c>
       <c r="D71" s="0" t="inlineStr">
@@ -2346,7 +2363,8 @@
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>철갑전사가 피해를 받을 때마다 4초 동안 방어력이 5% 증가하며 최대 4회 중첩. 다시 발동하면 지속시간 갱신</t>
+          <t xml:space="preserve">철갑전사가 피해를 받을 때마다 4초 동안 방어력이 5% 증가
+최대 4회 중첩되며 재발동 시 지속시간 갱신</t>
         </is>
       </c>
       <c r="D73" s="0" t="inlineStr">
@@ -2371,7 +2389,7 @@
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>아군 전사 클래스가 액티브 스킬 사용을 완료하면 자신 주변 반경 2.5의 적 최대 3명을 0.4초 동안 기절시킴</t>
+          <t xml:space="preserve">전사 계열 아군이 액티브 스킬 사용을 마치면 주변 반경 2.5 안의 적 최대 3명을 0.4초 동안 기절시킴</t>
         </is>
       </c>
       <c r="D74" s="0" t="inlineStr">
@@ -2396,7 +2414,7 @@
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>아군 마법사 클래스가 액티브 스킬 사용을 완료하면 자신 주변 반경 5의 적 최대 2명을 1초 동안 침묵시킴</t>
+          <t xml:space="preserve">마법사 계열 아군이 액티브 스킬 사용을 마치면 주변 반경 5 안의 적 최대 2명을 1초 동안 침묵시킴</t>
         </is>
       </c>
       <c r="D75" s="0" t="inlineStr">
@@ -2421,7 +2439,7 @@
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>빙결술사가 7초마다 자신 주변 반경 5의 적 최대 2명을 0.6초 동안 동결시킴</t>
+          <t xml:space="preserve">빙결술사가 7초마다 주변 반경 5 안의 적 최대 2명을 0.6초 동안 동결시킴</t>
         </is>
       </c>
       <c r="D76" s="0" t="inlineStr">
@@ -2446,7 +2464,9 @@
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>아군 전사 클래스가 피해를 줄 때마다 공격력이 5% 증가하며 최대 10회 중첩. 유닛이 유지되는 동안 지속되며 받는 피해가 25% 증가</t>
+          <t xml:space="preserve">전사 계열 아군이 피해를 줄 때마다 공격력이 5% 증가
+최대 10회 중첩되며 해당 유닛이 사라질 때까지 유지
+받는 피해는 항상 25% 증가</t>
         </is>
       </c>
       <c r="D77" s="0" t="inlineStr">
@@ -2471,7 +2491,8 @@
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>아군 궁수 클래스가 적을 처치하면 처치 위치 주변 반경 4의 적 최대 2명에게 공격력의 60%에 해당하는 물리 피해를 주는 투사체 발사. 공격력은 15% 감소</t>
+          <t xml:space="preserve">궁수 계열 아군이 적을 처치하면 처치한 적의 위치에서 반경 4 안의 적 최대 2명에게 투사체를 발사해 공격력의 60%만큼 물리 피해를 줌
+공격력은 15% 감소</t>
         </is>
       </c>
       <c r="D78" s="0" t="inlineStr">

</xml_diff>